<commit_message>
Task2: publish generated TCO, slide, C4 and use-case images
</commit_message>
<xml_diff>
--- a/Task2/tco-model.xlsx
+++ b/Task2/tco-model.xlsx
@@ -11,13 +11,14 @@
     <sheet name="A Монолит" sheetId="2" r:id="rId2"/>
     <sheet name="B Сервисы" sheetId="3" r:id="rId3"/>
     <sheet name="C CTO" sheetId="4" r:id="rId4"/>
+    <sheet name="Сценарии 50k 10M" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="90">
   <si>
     <t>Параметр</t>
   </si>
@@ -154,6 +155,18 @@
     <t>Все тарифы гипотетические, не договорные; input Task1 C-01/C-07.</t>
   </si>
   <si>
+    <t>Второй локальный контур NG/KE, USD/мес.</t>
+  </si>
+  <si>
+    <t>Внутристрановое резервирование, USD/мес.</t>
+  </si>
+  <si>
+    <t>Суммарное дополнительное размещение, USD/мес.</t>
+  </si>
+  <si>
+    <t>Статус: смета не подтверждена; обязательна проверка ЦОД NG/KE и CFO.</t>
+  </si>
+  <si>
     <t>A Монолит | TCO 5 лет (USD)</t>
   </si>
   <si>
@@ -232,7 +245,7 @@
     <t>TCO с условной стоимостью простоя</t>
   </si>
   <si>
-    <t>Сценарий 50k: неизменные 50k пользователей все 5 лет; B24 = difference in fixed overhead vs A.</t>
+    <t>B24 = разница фиксированных затрат относительно A (не сумма списаний); объём заказов на неё не влияет.</t>
   </si>
   <si>
     <t>Сценарий 10M: резерв B28 не включён в baseline; нужна проверка нагрузки и коммерческих тарифов.</t>
@@ -245,6 +258,36 @@
   </si>
   <si>
     <t>C CTO | TCO 5 лет (USD)</t>
+  </si>
+  <si>
+    <t>Сценарий</t>
+  </si>
+  <si>
+    <t>A Монолит</t>
+  </si>
+  <si>
+    <t>B Сервисы</t>
+  </si>
+  <si>
+    <t>C CTO</t>
+  </si>
+  <si>
+    <t>5-летняя фиксированная разница относительно A, USD</t>
+  </si>
+  <si>
+    <t>Сценарий: 50 000 пользователей в каждый год</t>
+  </si>
+  <si>
+    <t>Заказы в год при 2,4 заказа/пользователя</t>
+  </si>
+  <si>
+    <t>Сценарий: 10 млн пользователей, гипотеза, НЕ проверенная нагрузка</t>
+  </si>
+  <si>
+    <t>Условная стоимость миграции при 10 млн (не baseline)</t>
+  </si>
+  <si>
+    <t>Ни 50 тыс., ни 10 млн не являются фактическим прогнозом. Фиксированные затраты при 50 тыс. остаются, но не обязательно потеряны.</t>
   </si>
 </sst>
 </file>
@@ -607,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="37.7109375" customWidth="1"/>
@@ -932,6 +975,36 @@
     <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="2">
+        <f>SUM(B26:B27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -950,12 +1023,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>36</v>
@@ -1050,7 +1123,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B8" s="2">
         <f>2600*12*(1+'Допущения'!$B$7)^0</f>
@@ -1075,7 +1148,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2">
         <f>6*'Допущения'!$B$11*12*(1+'Допущения'!$B$8)^0</f>
@@ -1100,7 +1173,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B10" s="2">
         <f>B6*'Допущения'!$B$4</f>
@@ -1125,7 +1198,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B11" s="2">
         <f>B5*'Допущения'!$B$5</f>
@@ -1150,7 +1223,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2">
         <f>B5*'Допущения'!$B$6</f>
@@ -1175,7 +1248,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B13" s="2">
         <f>'Допущения'!$B$12</f>
@@ -1200,7 +1273,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B14" s="2">
         <v>6000</v>
@@ -1220,7 +1293,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B15" s="2">
         <f>SUM(B8:B14)</f>
@@ -1245,7 +1318,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B16" s="2">
         <f>B8+B9+B13+B14</f>
@@ -1270,7 +1343,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B17" s="2">
         <f>B15/B5</f>
@@ -1295,7 +1368,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B18" s="2">
         <f>B16/B5</f>
@@ -1320,7 +1393,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B19" s="2">
         <f>B15/(1+'Допущения'!$B$10)^1</f>
@@ -1345,7 +1418,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B21" s="2">
         <f>SUM(B15:F15)</f>
@@ -1354,7 +1427,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B22" s="2">
         <f>SUM(B19:F19)</f>
@@ -1363,7 +1436,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B23" s="2">
         <f>B21/SUM(B5:F5)</f>
@@ -1372,16 +1445,16 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B24" s="2">
-        <f>SUM(B8:F9)+SUM(B13:F14)-SUM(31200*(1+'Допущения'!$B$7)^0,31200*(1+'Допущения'!$B$7)^1,31200*(1+'Допущения'!$B$7)^2,31200*(1+'Допущения'!$B$7)^3,31200*(1+'Допущения'!$B$7)^4)-SUM(252000*(1+'Допущения'!$B$8)^0,252000*(1+'Допущения'!$B$8)^1,252000*(1+'Допущения'!$B$8)^2,252000*(1+'Допущения'!$B$8)^3,252000*(1+'Допущения'!$B$8)^4)-20000-4*7000-6000</f>
+        <f>SUM(B8:F9)+SUM(B13:F14)-SUM('A Монолит'!B8:F9)-SUM('A Монолит'!B13:F14)</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B25" s="2">
         <f>B8/12</f>
@@ -1390,7 +1463,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B26">
         <f>IF(B25&lt;='Допущения'!$B$16,1,0)</f>
@@ -1399,7 +1472,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B27">
         <v>6</v>
@@ -1407,7 +1480,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B28">
         <v>50000</v>
@@ -1415,7 +1488,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B30" s="2">
         <f>'Допущения'!$B$15</f>
@@ -1440,7 +1513,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B31" s="2">
         <f>(1-B30)*365*24*60</f>
@@ -1465,7 +1538,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B32" s="2">
         <f>B31*'Допущения'!$B$14</f>
@@ -1490,7 +1563,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B33" s="2">
         <f>B15+B32</f>
@@ -1515,17 +1588,17 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1544,12 +1617,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>36</v>
@@ -1644,7 +1717,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B8" s="2">
         <f>4700*12*(1+'Допущения'!$B$7)^0</f>
@@ -1669,7 +1742,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2">
         <f>9*'Допущения'!$B$11*12*(1+'Допущения'!$B$8)^0</f>
@@ -1694,7 +1767,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B10" s="2">
         <f>B6*'Допущения'!$B$4</f>
@@ -1719,7 +1792,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B11" s="2">
         <f>B5*'Допущения'!$B$5</f>
@@ -1744,7 +1817,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2">
         <f>B5*'Допущения'!$B$6</f>
@@ -1769,7 +1842,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B13" s="2">
         <f>'Допущения'!$B$12</f>
@@ -1794,7 +1867,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B14" s="2">
         <v>18000</v>
@@ -1814,7 +1887,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B15" s="2">
         <f>SUM(B8:B14)</f>
@@ -1839,7 +1912,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B16" s="2">
         <f>B8+B9+B13+B14</f>
@@ -1864,7 +1937,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B17" s="2">
         <f>B15/B5</f>
@@ -1889,7 +1962,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B18" s="2">
         <f>B16/B5</f>
@@ -1914,7 +1987,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B19" s="2">
         <f>B15/(1+'Допущения'!$B$10)^1</f>
@@ -1939,7 +2012,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B21" s="2">
         <f>SUM(B15:F15)</f>
@@ -1948,7 +2021,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B22" s="2">
         <f>SUM(B19:F19)</f>
@@ -1957,7 +2030,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B23" s="2">
         <f>B21/SUM(B5:F5)</f>
@@ -1966,16 +2039,16 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B24" s="2">
-        <f>SUM(B8:F9)+SUM(B13:F14)-SUM(31200*(1+'Допущения'!$B$7)^0,31200*(1+'Допущения'!$B$7)^1,31200*(1+'Допущения'!$B$7)^2,31200*(1+'Допущения'!$B$7)^3,31200*(1+'Допущения'!$B$7)^4)-SUM(252000*(1+'Допущения'!$B$8)^0,252000*(1+'Допущения'!$B$8)^1,252000*(1+'Допущения'!$B$8)^2,252000*(1+'Допущения'!$B$8)^3,252000*(1+'Допущения'!$B$8)^4)-20000-4*7000-6000</f>
+        <f>SUM(B8:F9)+SUM(B13:F14)-SUM('A Монолит'!B8:F9)-SUM('A Монолит'!B13:F14)</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B25" s="2">
         <f>B8/12</f>
@@ -1984,7 +2057,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B26">
         <f>IF(B25&lt;='Допущения'!$B$16,1,0)</f>
@@ -1993,7 +2066,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B27">
         <v>9</v>
@@ -2001,7 +2074,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B28">
         <v>100000</v>
@@ -2009,7 +2082,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B30" s="2">
         <f>'Допущения'!$B$15</f>
@@ -2034,7 +2107,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B31" s="2">
         <f>(1-B30)*365*24*60</f>
@@ -2059,7 +2132,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B32" s="2">
         <f>B31*'Допущения'!$B$14</f>
@@ -2084,7 +2157,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B33" s="2">
         <f>B15+B32</f>
@@ -2109,17 +2182,17 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -2138,12 +2211,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>36</v>
@@ -2238,7 +2311,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B8" s="2">
         <f>18500*12*(1+'Допущения'!$B$7)^0</f>
@@ -2263,7 +2336,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2">
         <f>18*'Допущения'!$B$11*12*(1+'Допущения'!$B$8)^0</f>
@@ -2288,7 +2361,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B10" s="2">
         <f>B6*'Допущения'!$B$4</f>
@@ -2313,7 +2386,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B11" s="2">
         <f>B5*'Допущения'!$B$5</f>
@@ -2338,7 +2411,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2">
         <f>B5*'Допущения'!$B$6</f>
@@ -2363,7 +2436,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B13" s="2">
         <f>'Допущения'!$B$12</f>
@@ -2388,7 +2461,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B14" s="2">
         <v>80000</v>
@@ -2408,7 +2481,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B15" s="2">
         <f>SUM(B8:B14)</f>
@@ -2433,7 +2506,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B16" s="2">
         <f>B8+B9+B13+B14</f>
@@ -2458,7 +2531,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B17" s="2">
         <f>B15/B5</f>
@@ -2483,7 +2556,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B18" s="2">
         <f>B16/B5</f>
@@ -2508,7 +2581,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B19" s="2">
         <f>B15/(1+'Допущения'!$B$10)^1</f>
@@ -2533,7 +2606,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B21" s="2">
         <f>SUM(B15:F15)</f>
@@ -2542,7 +2615,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B22" s="2">
         <f>SUM(B19:F19)</f>
@@ -2551,7 +2624,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B23" s="2">
         <f>B21/SUM(B5:F5)</f>
@@ -2560,16 +2633,16 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B24" s="2">
-        <f>SUM(B8:F9)+SUM(B13:F14)-SUM(31200*(1+'Допущения'!$B$7)^0,31200*(1+'Допущения'!$B$7)^1,31200*(1+'Допущения'!$B$7)^2,31200*(1+'Допущения'!$B$7)^3,31200*(1+'Допущения'!$B$7)^4)-SUM(252000*(1+'Допущения'!$B$8)^0,252000*(1+'Допущения'!$B$8)^1,252000*(1+'Допущения'!$B$8)^2,252000*(1+'Допущения'!$B$8)^3,252000*(1+'Допущения'!$B$8)^4)-20000-4*7000-6000</f>
+        <f>SUM(B8:F9)+SUM(B13:F14)-SUM('A Монолит'!B8:F9)-SUM('A Монолит'!B13:F14)</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B25" s="2">
         <f>B8/12</f>
@@ -2578,7 +2651,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B26">
         <f>IF(B25&lt;='Допущения'!$B$16,1,0)</f>
@@ -2587,7 +2660,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B27">
         <v>18</v>
@@ -2595,7 +2668,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B28">
         <v>250000</v>
@@ -2603,7 +2676,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B30" s="2">
         <f>'Допущения'!$B$15</f>
@@ -2628,7 +2701,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B31" s="2">
         <f>(1-B30)*365*24*60</f>
@@ -2653,7 +2726,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B32" s="2">
         <f>B31*'Допущения'!$B$14</f>
@@ -2678,7 +2751,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B33" s="2">
         <f>B15+B32</f>
@@ -2703,17 +2776,112 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="51.7109375" customWidth="1"/>
+    <col min="2" max="4" width="25.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="2">
+        <f>'A Монолит'!B24</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <f>'B Сервисы'!B24</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="2">
+        <f>'C CTO'!B24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4">
+        <f>50000*'Допущения'!B3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6">
+        <f>10000000*'Допущения'!B3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="2">
+        <f>'A Монолит'!B28</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="2">
+        <f>'B Сервисы'!B28</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="2">
+        <f>'C CTO'!B28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="3" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>